<commit_message>
Rename the app to Finance Dojo
The window title, sidebar, exports, docs, exe, zip and build scripts now use
the Finance Dojo name. The per-user data folder becomes %APPDATA%\Finance_Dojo;
progress in the old Finance_Commercial_Training folder is copied over on first
start and the original is left in place.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011X2bGRbbM1wG3sUYL2koaP
</commit_message>
<xml_diff>
--- a/workbooks/ANSWER_KEY_Workbook_Aurelia_Grand.xlsx
+++ b/workbooks/ANSWER_KEY_Workbook_Aurelia_Grand.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Exercises" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Raw Data" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Assumptions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exercises" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -522,7 +522,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fictional training data generated by Finance &amp; Commercial Training Simulator. Not real company or industry data.</t>
+          <t>Fictional training data generated by Finance Dojo. Not real company or industry data.</t>
         </is>
       </c>
     </row>

</xml_diff>